<commit_message>
Add the demo video script, and correct the provenance-cell count
A 2:45 shot list with what to show, what to say, and the timing. Every
number it asks you to speak was checked against a live run first -- the
provenance-cell figure had drifted to 26,627 and is corrected in the
script, the deck, the README and the brief.

The script's own rule: never claim a number the screen is not showing at
that moment.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/out_foreign/delivery.xlsx
+++ b/data/out_foreign/delivery.xlsx
@@ -1330,7 +1330,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco Products, Inc. Satco®, Light Bulb, Incan, S4724, Electrical</t>
+          <t xml:space="preserve">Satco Products, Inc. Satco, Light Bulb, S4724, 4 W, 2700 K, Candelabra Base</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -1340,17 +1340,17 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Incan S4724 Light Bulb, 4 W, 2700 K, Candelabra Base, 4</t>
+          <t xml:space="preserve">Satco® S4724 Light Bulb, 4 W, 2700 K, Candelabra Base, 4</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Light Bulb, Incan, 4 W, 2700 K, Candelabra Base, 4</t>
+          <t xml:space="preserve">Satco® Light Bulb, 4 W, 2700 K, Candelabra Base, 4</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incan Light Bulb, 4 W, 2700 K, Candelabra Base, 4</t>
+          <t xml:space="preserve">Light Bulb, 4 W, 2700 K, Candelabra Base, 4</t>
         </is>
       </c>
       <c r="BC2" t="inlineStr">
@@ -1360,60 +1360,50 @@
       </c>
       <c r="BD2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Wattage</t>
         </is>
       </c>
       <c r="BE2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incan</t>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W</t>
         </is>
       </c>
       <c r="BG2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wattage</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BH2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2700</t>
         </is>
       </c>
       <c r="BI2" t="inlineStr">
         <is>
-          <t xml:space="preserve">W</t>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BJ2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Base Type</t>
         </is>
       </c>
       <c r="BK2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2700</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">Candelabra Base</t>
         </is>
       </c>
       <c r="BM2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base Type</t>
+          <t xml:space="preserve">Pack Quantity</t>
         </is>
       </c>
       <c r="BN2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Candelabra Base</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pack Quantity</t>
-        </is>
-      </c>
-      <c r="BQ2" t="inlineStr">
         <is>
           <t xml:space="preserve">4</t>
         </is>
@@ -1482,27 +1472,27 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stanley Black &amp; Decker DEWALT®, Die Grinder, DCG420B, Tools, Power Tools</t>
+          <t xml:space="preserve">Stanley Black &amp; Decker DEWALT, Die Grinder, DCG420B, 20 V</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIE GRINDER 20V NO</t>
+          <t xml:space="preserve">DIE GRINDER 20V</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEWALT® DCG420B Die Grinder, 20 V, No</t>
+          <t xml:space="preserve">DEWALT® DCG420B Die Grinder, 20 V</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEWALT® Die Grinder, 20 V, No</t>
+          <t xml:space="preserve">DEWALT® Die Grinder, 20 V</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Die Grinder, 20 V, No</t>
+          <t xml:space="preserve">Die Grinder, 20 V</t>
         </is>
       </c>
       <c r="BC3" t="inlineStr">
@@ -1599,7 +1589,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Signify Holding Philips®, Light Bulb, Led, 571513, Lighting, Electrical</t>
+          <t xml:space="preserve">Signify Holding Philips, Light Bulb, 571513, 2700 K, LED, Medium Base</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -1609,17 +1599,17 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Led 571513 Light Bulb, 2700 K, LED, Medium Base</t>
+          <t xml:space="preserve">Philips® 571513 Light Bulb, 2700 K, LED, Medium Base</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Light Bulb, Led, 2700 K, LED, Medium Base</t>
+          <t xml:space="preserve">Philips® Light Bulb, 2700 K, LED, Medium Base</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led Light Bulb, 2700 K, LED, Medium Base</t>
+          <t xml:space="preserve">Light Bulb, 2700 K, LED, Medium Base</t>
         </is>
       </c>
       <c r="BC4" t="inlineStr">
@@ -1629,45 +1619,35 @@
       </c>
       <c r="BD4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BE4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led</t>
+          <t xml:space="preserve">2700</t>
+        </is>
+      </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BG4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Lamp Type</t>
         </is>
       </c>
       <c r="BH4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2700</t>
-        </is>
-      </c>
-      <c r="BI4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">LED</t>
         </is>
       </c>
       <c r="BJ4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamp Type</t>
+          <t xml:space="preserve">Base Type</t>
         </is>
       </c>
       <c r="BK4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LED</t>
-        </is>
-      </c>
-      <c r="BM4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Base Type</t>
-        </is>
-      </c>
-      <c r="BN4" t="inlineStr">
         <is>
           <t xml:space="preserve">Medium Base</t>
         </is>
@@ -1736,32 +1716,32 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee Tool Milwaukee®, Rachet, 3052-20, Tools, Hand Tools</t>
+          <t xml:space="preserve">Milwaukee Tool Milwaukee, Fuel Rachet, 3052-20, 1/4 in, M12</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t xml:space="preserve">RACHET 1/4IN M12</t>
+          <t xml:space="preserve">FUEL RACHET 1/4IN M12</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee® 3052-20 Rachet, 1/4 in, M12</t>
+          <t xml:space="preserve">Milwaukee® 3052-20 Fuel Rachet, 1/4 in, M12</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee® Rachet, 1/4 in, M12</t>
+          <t xml:space="preserve">Milwaukee® Fuel Rachet, 1/4 in, M12</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rachet, 1/4 in, M12</t>
+          <t xml:space="preserve">Fuel Rachet, 1/4 in, M12</t>
         </is>
       </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rachet</t>
+          <t xml:space="preserve">Fuel Rachet</t>
         </is>
       </c>
       <c r="BD5" t="inlineStr">
@@ -1853,67 +1833,67 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita U.S.A., Inc. Makita®, Tool, Recip Saw, XRJ08Z, Tools, Power Tools</t>
+          <t xml:space="preserve">Makita U.S.A., Inc. Makita, Recip Saw, XRJ08Z, 18 V, 18V, Bare Tool</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOOL 18V 18V</t>
+          <t xml:space="preserve">RECIP SAW 18V 18V BARE TOOL</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita® Recip Saw XRJ08Z Tool, 18 V, 18V</t>
+          <t xml:space="preserve">Makita® XRJ08Z Recip Saw, 18 V, 18V, Bare Tool</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita® Tool, Recip Saw, 18 V, 18V</t>
+          <t xml:space="preserve">Makita® Recip Saw, 18 V, 18V, Bare Tool</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recip Saw Tool, 18 V, 18V</t>
+          <t xml:space="preserve">Recip Saw, 18 V, 18V, Bare Tool</t>
         </is>
       </c>
       <c r="BC6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tool</t>
+          <t xml:space="preserve">Recip Saw</t>
         </is>
       </c>
       <c r="BD6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Voltage Rating</t>
         </is>
       </c>
       <c r="BE6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recip Saw</t>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
         </is>
       </c>
       <c r="BG6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voltage Rating</t>
+          <t xml:space="preserve">Battery Platform</t>
         </is>
       </c>
       <c r="BH6" t="inlineStr">
         <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="BI6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">V</t>
+          <t xml:space="preserve">18V</t>
         </is>
       </c>
       <c r="BJ6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Battery Platform</t>
+          <t xml:space="preserve">Configuration</t>
         </is>
       </c>
       <c r="BK6" t="inlineStr">
         <is>
-          <t xml:space="preserve">18V</t>
+          <t xml:space="preserve">Bare Tool</t>
         </is>
       </c>
       <c r="HA6" t="inlineStr">
@@ -1980,50 +1960,40 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee Tool Milwaukee®, Blower, Brushless Precision, 0887-20</t>
+          <t xml:space="preserve">Milwaukee Tool Milwaukee, Precision Blower, 0887-20, M18</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOWER M18</t>
+          <t xml:space="preserve">PRECISION BLOWER M18</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee® Brushless Precision 0887-20 Blower, M18</t>
+          <t xml:space="preserve">Milwaukee® 0887-20 Precision Blower, M18</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee® Blower, Brushless Precision, M18</t>
+          <t xml:space="preserve">Milwaukee® Precision Blower, M18</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brushless Precision Blower, M18</t>
+          <t xml:space="preserve">Precision Blower, M18</t>
         </is>
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blower</t>
+          <t xml:space="preserve">Precision Blower</t>
         </is>
       </c>
       <c r="BD7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Battery Platform</t>
         </is>
       </c>
       <c r="BE7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Brushless Precision</t>
-        </is>
-      </c>
-      <c r="BG7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Battery Platform</t>
-        </is>
-      </c>
-      <c r="BH7" t="inlineStr">
         <is>
           <t xml:space="preserve">M18</t>
         </is>
@@ -2092,7 +2062,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Signify Holding Philips®, Light Bulb, Led, 565374, Electrical</t>
+          <t xml:space="preserve">Signify Holding Philips, Light Bulb, 565374, 75 W, 2700 K, LED</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -2102,17 +2072,17 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Led 565374 Light Bulb, 75 W, 2700 K, LED, A19</t>
+          <t xml:space="preserve">Philips® 565374 Light Bulb, 75 W, 2700 K, LED, A19</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Light Bulb, Led, 75 W, 2700 K, LED, A19, Medium Base, 4</t>
+          <t xml:space="preserve">Philips® Light Bulb, 75 W, 2700 K, LED, A19, Medium Base, 4</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led Light Bulb, 75 W, 2700 K, LED, A19</t>
+          <t xml:space="preserve">Light Bulb, 75 W, 2700 K, LED, A19</t>
         </is>
       </c>
       <c r="BC8" t="inlineStr">
@@ -2122,80 +2092,70 @@
       </c>
       <c r="BD8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Wattage</t>
         </is>
       </c>
       <c r="BE8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led</t>
+          <t xml:space="preserve">75</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W</t>
         </is>
       </c>
       <c r="BG8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wattage</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BH8" t="inlineStr">
         <is>
-          <t xml:space="preserve">75</t>
+          <t xml:space="preserve">2700</t>
         </is>
       </c>
       <c r="BI8" t="inlineStr">
         <is>
-          <t xml:space="preserve">W</t>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BJ8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Lamp Type</t>
         </is>
       </c>
       <c r="BK8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2700</t>
-        </is>
-      </c>
-      <c r="BL8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">LED</t>
         </is>
       </c>
       <c r="BM8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamp Type</t>
+          <t xml:space="preserve">Bulb Shape</t>
         </is>
       </c>
       <c r="BN8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED</t>
+          <t xml:space="preserve">A19</t>
         </is>
       </c>
       <c r="BP8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bulb Shape</t>
+          <t xml:space="preserve">Base Type</t>
         </is>
       </c>
       <c r="BQ8" t="inlineStr">
         <is>
-          <t xml:space="preserve">A19</t>
+          <t xml:space="preserve">Medium Base</t>
         </is>
       </c>
       <c r="BS8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base Type</t>
+          <t xml:space="preserve">Pack Quantity</t>
         </is>
       </c>
       <c r="BT8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Medium Base</t>
-        </is>
-      </c>
-      <c r="BV8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pack Quantity</t>
-        </is>
-      </c>
-      <c r="BW8" t="inlineStr">
         <is>
           <t xml:space="preserve">4</t>
         </is>
@@ -2264,7 +2224,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco Products, Inc. Satco®, Light Bulb, Incan, S3797, Electrical</t>
+          <t xml:space="preserve">Satco Products, Inc. Satco, Light Bulb, S3797, 4 W, 2700 K, Candelabra Base</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -2274,17 +2234,17 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Incan S3797 Light Bulb, 4 W, 2700 K, Candelabra Base, 2</t>
+          <t xml:space="preserve">Satco® S3797 Light Bulb, 4 W, 2700 K, Candelabra Base, 2</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Light Bulb, Incan, 4 W, 2700 K, Candelabra Base, 2</t>
+          <t xml:space="preserve">Satco® Light Bulb, 4 W, 2700 K, Candelabra Base, 2</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incan Light Bulb, 4 W, 2700 K, Candelabra Base, 2</t>
+          <t xml:space="preserve">Light Bulb, 4 W, 2700 K, Candelabra Base, 2</t>
         </is>
       </c>
       <c r="BC9" t="inlineStr">
@@ -2294,60 +2254,50 @@
       </c>
       <c r="BD9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Wattage</t>
         </is>
       </c>
       <c r="BE9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incan</t>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W</t>
         </is>
       </c>
       <c r="BG9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wattage</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BH9" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2700</t>
         </is>
       </c>
       <c r="BI9" t="inlineStr">
         <is>
-          <t xml:space="preserve">W</t>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BJ9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Base Type</t>
         </is>
       </c>
       <c r="BK9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2700</t>
-        </is>
-      </c>
-      <c r="BL9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">Candelabra Base</t>
         </is>
       </c>
       <c r="BM9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base Type</t>
+          <t xml:space="preserve">Pack Quantity</t>
         </is>
       </c>
       <c r="BN9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Candelabra Base</t>
-        </is>
-      </c>
-      <c r="BP9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pack Quantity</t>
-        </is>
-      </c>
-      <c r="BQ9" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
@@ -2416,7 +2366,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Signify Holding Philips®, Light Bulb, Led, 565622, Electrical</t>
+          <t xml:space="preserve">Signify Holding Philips, Light Bulb, 565622, 60 W, 2000 K, LED</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -2426,17 +2376,17 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Led 565622 Light Bulb, 60 W, 2000 K, LED, Medium Base</t>
+          <t xml:space="preserve">Philips® 565622 Light Bulb, 60 W, 2000 K, LED, Medium Base</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Light Bulb, Led, 60 W, 2000 K, LED, Medium Base</t>
+          <t xml:space="preserve">Philips® Light Bulb, 60 W, 2000 K, LED, Medium Base</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led Light Bulb, 60 W, 2000 K, LED, Medium Base</t>
+          <t xml:space="preserve">Light Bulb, 60 W, 2000 K, LED, Medium Base</t>
         </is>
       </c>
       <c r="BC10" t="inlineStr">
@@ -2446,60 +2396,50 @@
       </c>
       <c r="BD10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Wattage</t>
         </is>
       </c>
       <c r="BE10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led</t>
+          <t xml:space="preserve">60</t>
+        </is>
+      </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W</t>
         </is>
       </c>
       <c r="BG10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wattage</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BH10" t="inlineStr">
         <is>
-          <t xml:space="preserve">60</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="BI10" t="inlineStr">
         <is>
-          <t xml:space="preserve">W</t>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BJ10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Lamp Type</t>
         </is>
       </c>
       <c r="BK10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
-        </is>
-      </c>
-      <c r="BL10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">LED</t>
         </is>
       </c>
       <c r="BM10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamp Type</t>
+          <t xml:space="preserve">Base Type</t>
         </is>
       </c>
       <c r="BN10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LED</t>
-        </is>
-      </c>
-      <c r="BP10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Base Type</t>
-        </is>
-      </c>
-      <c r="BQ10" t="inlineStr">
         <is>
           <t xml:space="preserve">Medium Base</t>
         </is>
@@ -2568,32 +2508,32 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita U.S.A., Inc. Makita®, Impact, XLT05Z, Tools, Power Tools</t>
+          <t xml:space="preserve">Makita U.S.A., Inc. Makita, Angle Impact, XLT05Z, 1/2 in, 18 V</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPACT 18V 1/2IN 18V</t>
+          <t xml:space="preserve">ANGLE IMPACT 18V 1/2IN 18V</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita® XLT05Z Impact, 1/2 in, 18 V, 18V</t>
+          <t xml:space="preserve">Makita® XLT05Z Angle Impact, 1/2 in, 18 V, 18V</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita® Impact, 1/2 in, 18 V, 18V</t>
+          <t xml:space="preserve">Makita® Angle Impact, 1/2 in, 18 V, 18V</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impact, 1/2 in, 18 V, 18V</t>
+          <t xml:space="preserve">Angle Impact, 1/2 in, 18 V, 18V</t>
         </is>
       </c>
       <c r="BC11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impact</t>
+          <t xml:space="preserve">Angle Impact</t>
         </is>
       </c>
       <c r="BD11" t="inlineStr">
@@ -2700,32 +2640,32 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leviton Manufacturing Co., Inc. Leviton®, Outlet, R02-D215P-1RW</t>
+          <t xml:space="preserve">Leviton Manufacturing Co., Inc. Leviton, Mini Outlet, R02-D215P-1RW</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTLET WH 15A</t>
+          <t xml:space="preserve">MINI OUTLET WH 15A</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leviton® R02-D215P-1RW Outlet, 15 A, White</t>
+          <t xml:space="preserve">Leviton® R02-D215P-1RW Mini Outlet, 15 A, White</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leviton® Outlet, 15 A, White</t>
+          <t xml:space="preserve">Leviton® Mini Outlet, 15 A, White</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outlet, 15 A, White</t>
+          <t xml:space="preserve">Mini Outlet, 15 A, White</t>
         </is>
       </c>
       <c r="BC12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outlet</t>
+          <t xml:space="preserve">Mini Outlet</t>
         </is>
       </c>
       <c r="BD12" t="inlineStr">
@@ -2817,27 +2757,27 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex Company, Inc. Trex®, Decking, Salt Transcend Lineage, 1513712</t>
+          <t xml:space="preserve">Trex Company, Inc. Trex, Decking, Transcend Lineage, 1513712</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECKING 1IN X 6IN 20FT</t>
+          <t xml:space="preserve">DECKING 1IN X 6IN 20FT GRVD</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Salt Transcend Lineage 1513712 Decking, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Trex® Transcend Lineage 1513712 Decking, 1 in x 6 in, 20 ft, Grooved</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Decking, Salt Transcend Lineage, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Trex® Decking, Transcend Lineage, 1 in x 6 in, 20 ft, Grooved</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salt Transcend Lineage Decking, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Transcend Lineage Decking, 1 in x 6 in, 20 ft, Grooved</t>
         </is>
       </c>
       <c r="BC13" t="inlineStr">
@@ -2872,12 +2812,22 @@
       </c>
       <c r="BJ13" t="inlineStr">
         <is>
+          <t xml:space="preserve">Edge Profile</t>
+        </is>
+      </c>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grooved</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
           <t xml:space="preserve">Series</t>
         </is>
       </c>
-      <c r="BK13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Salt Transcend Lineage</t>
+      <c r="BN13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transcend Lineage</t>
         </is>
       </c>
       <c r="HA13" t="inlineStr">
@@ -2944,27 +2894,27 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex Company, Inc. Trex®, Decking, Hatteras Transcend Lineage, 1513707</t>
+          <t xml:space="preserve">Trex Company, Inc. Trex, Decking, Transcend Lineage, 1513707</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECKING 1IN X 6IN 20FT</t>
+          <t xml:space="preserve">DECKING 1IN X 6IN 20FT GRVD</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Hatteras Transcend Lineage 1513707 Decking, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Trex® Transcend Lineage 1513707 Decking, 1 in x 6 in, 20 ft, Grooved</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Decking, Hatteras Transcend Lineage, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Trex® Decking, Transcend Lineage, 1 in x 6 in, 20 ft, Grooved</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hatteras Transcend Lineage Decking, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Transcend Lineage Decking, 1 in x 6 in, 20 ft, Grooved</t>
         </is>
       </c>
       <c r="BC14" t="inlineStr">
@@ -2999,12 +2949,22 @@
       </c>
       <c r="BJ14" t="inlineStr">
         <is>
+          <t xml:space="preserve">Edge Profile</t>
+        </is>
+      </c>
+      <c r="BK14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grooved</t>
+        </is>
+      </c>
+      <c r="BM14" t="inlineStr">
+        <is>
           <t xml:space="preserve">Series</t>
         </is>
       </c>
-      <c r="BK14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hatteras Transcend Lineage</t>
+      <c r="BN14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transcend Lineage</t>
         </is>
       </c>
       <c r="HA14" t="inlineStr">
@@ -3071,7 +3031,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita U.S.A., Inc. Makita®, Finish Nailer, XNB05Z, Tools, Power Tools</t>
+          <t xml:space="preserve">Makita U.S.A., Inc. Makita, Finish Nailer, XNB05Z, 2-1/2 in, 18 V</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -3218,7 +3178,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Signify Holding Philips®, Light Bulb, Led, 566687, Electrical</t>
+          <t xml:space="preserve">Signify Holding Philips, Light Bulb, 566687, 60 W, 2700 K, LED</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -3228,17 +3188,17 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Led 566687 Light Bulb, 60 W, 2700 K, LED, Candelabra Base</t>
+          <t xml:space="preserve">Philips® 566687 Light Bulb, 60 W, 2700 K, LED, Candelabra Base</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Light Bulb, Led, 60 W, 2700 K, LED, Candelabra Base, 3</t>
+          <t xml:space="preserve">Philips® Light Bulb, 60 W, 2700 K, LED, Candelabra Base, 3</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led Light Bulb, 60 W, 2700 K, LED, Candelabra Base</t>
+          <t xml:space="preserve">Light Bulb, 60 W, 2700 K, LED, Candelabra Base</t>
         </is>
       </c>
       <c r="BC16" t="inlineStr">
@@ -3248,70 +3208,60 @@
       </c>
       <c r="BD16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Wattage</t>
         </is>
       </c>
       <c r="BE16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led</t>
+          <t xml:space="preserve">60</t>
+        </is>
+      </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W</t>
         </is>
       </c>
       <c r="BG16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wattage</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BH16" t="inlineStr">
         <is>
-          <t xml:space="preserve">60</t>
+          <t xml:space="preserve">2700</t>
         </is>
       </c>
       <c r="BI16" t="inlineStr">
         <is>
-          <t xml:space="preserve">W</t>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BJ16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Lamp Type</t>
         </is>
       </c>
       <c r="BK16" t="inlineStr">
         <is>
-          <t xml:space="preserve">2700</t>
-        </is>
-      </c>
-      <c r="BL16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">LED</t>
         </is>
       </c>
       <c r="BM16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamp Type</t>
+          <t xml:space="preserve">Base Type</t>
         </is>
       </c>
       <c r="BN16" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED</t>
+          <t xml:space="preserve">Candelabra Base</t>
         </is>
       </c>
       <c r="BP16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base Type</t>
+          <t xml:space="preserve">Pack Quantity</t>
         </is>
       </c>
       <c r="BQ16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Candelabra Base</t>
-        </is>
-      </c>
-      <c r="BS16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pack Quantity</t>
-        </is>
-      </c>
-      <c r="BT16" t="inlineStr">
         <is>
           <t xml:space="preserve">3</t>
         </is>
@@ -3380,7 +3330,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Signify Holding Philips®, Light Bulb, Led, 576397, Electrical</t>
+          <t xml:space="preserve">Signify Holding Philips, Light Bulb, 576397, 5000 K, LED, A23</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -3390,17 +3340,17 @@
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Led 576397 Light Bulb, 5000 K, LED, A23</t>
+          <t xml:space="preserve">Philips® 576397 Light Bulb, 5000 K, LED, A23</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Light Bulb, Led, 5000 K, LED, A23</t>
+          <t xml:space="preserve">Philips® Light Bulb, 5000 K, LED, A23</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led Light Bulb, 5000 K, LED, A23</t>
+          <t xml:space="preserve">Light Bulb, 5000 K, LED, A23</t>
         </is>
       </c>
       <c r="BC17" t="inlineStr">
@@ -3410,45 +3360,35 @@
       </c>
       <c r="BD17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BE17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led</t>
+          <t xml:space="preserve">5000</t>
+        </is>
+      </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BG17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Lamp Type</t>
         </is>
       </c>
       <c r="BH17" t="inlineStr">
         <is>
-          <t xml:space="preserve">5000</t>
-        </is>
-      </c>
-      <c r="BI17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">LED</t>
         </is>
       </c>
       <c r="BJ17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamp Type</t>
+          <t xml:space="preserve">Bulb Shape</t>
         </is>
       </c>
       <c r="BK17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LED</t>
-        </is>
-      </c>
-      <c r="BM17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bulb Shape</t>
-        </is>
-      </c>
-      <c r="BN17" t="inlineStr">
         <is>
           <t xml:space="preserve">A23</t>
         </is>
@@ -3517,12 +3457,12 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t xml:space="preserve">LG Electronics LG®, Range, Elec BS, LSEL6333ZE, Appliances, Large Appliances</t>
+          <t xml:space="preserve">LG Electronics LG, Range, Elec BS, LSEL6333ZE, 30 in</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t xml:space="preserve">RANGE 30IN YES</t>
+          <t xml:space="preserve">RANGE 30IN LSEL6333ZE</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -3532,7 +3472,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t xml:space="preserve">LG® Range, Elec BS, 30 in, Yes</t>
+          <t xml:space="preserve">LG® Range, Elec BS, 30 in</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
@@ -3644,50 +3584,40 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE Appliances Café®, Machine, Auto Espresso, C7CEBBS4RW3, Appliances</t>
+          <t xml:space="preserve">GE Appliances Café, Espresso Machine, C7CEBBS4RW3, White</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t xml:space="preserve">MACHINE WH</t>
+          <t xml:space="preserve">ESPRESSO MACHINE WH</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Café® Auto Espresso C7CEBBS4RW3 Machine, White</t>
+          <t xml:space="preserve">Café® C7CEBBS4RW3 Espresso Machine, White</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Café® Machine, Auto Espresso, White</t>
+          <t xml:space="preserve">Café® Espresso Machine, White</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auto Espresso Machine, White</t>
+          <t xml:space="preserve">Espresso Machine, White</t>
         </is>
       </c>
       <c r="BC19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine</t>
+          <t xml:space="preserve">Espresso Machine</t>
         </is>
       </c>
       <c r="BD19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Color</t>
         </is>
       </c>
       <c r="BE19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Auto Espresso</t>
-        </is>
-      </c>
-      <c r="BG19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Color</t>
-        </is>
-      </c>
-      <c r="BH19" t="inlineStr">
         <is>
           <t xml:space="preserve">White</t>
         </is>
@@ -3756,12 +3686,12 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kreg Tool Company Kreg®, Drill, Ionic Compact, KPTDR050A, Tools</t>
+          <t xml:space="preserve">Kreg Tool Company Kreg, Drill, Ionic Compact, KPTDR050A, 20 V</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t xml:space="preserve">DRILL 20V</t>
+          <t xml:space="preserve">DRILL 20V KPTDR050A</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
@@ -3873,27 +3803,27 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex Company, Inc. Trex®, Decking, Salt Sq Edge Transcend Lineage, 1513708</t>
+          <t xml:space="preserve">Trex Company, Inc. Trex, Decking, Transcend Lineage, 1513708</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECKING 1IN X 6IN 16FT</t>
+          <t xml:space="preserve">DECKING 1IN X 6IN 16FT SQ EDG</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Salt Sq Edge Transcend Lineage 1513708 Decking, 1 in x 6 in, 16 ft</t>
+          <t xml:space="preserve">Trex® Transcend Lineage 1513708 Decking, 1 in x 6 in, 16 ft, Square Edge</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Decking, Salt Sq Edge Transcend Lineage, 1 in x 6 in, 16 ft</t>
+          <t xml:space="preserve">Trex® Decking, Transcend Lineage, 1 in x 6 in, 16 ft, Square Edge</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salt Sq Edge Transcend Lineage Decking, 1 in x 6 in, 16 ft</t>
+          <t xml:space="preserve">Transcend Lineage Decking, 1 in x 6 in, 16 ft, Square Edge</t>
         </is>
       </c>
       <c r="BC21" t="inlineStr">
@@ -3928,12 +3858,22 @@
       </c>
       <c r="BJ21" t="inlineStr">
         <is>
+          <t xml:space="preserve">Edge Profile</t>
+        </is>
+      </c>
+      <c r="BK21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square Edge</t>
+        </is>
+      </c>
+      <c r="BM21" t="inlineStr">
+        <is>
           <t xml:space="preserve">Series</t>
         </is>
       </c>
-      <c r="BK21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Salt Sq Edge Transcend Lineage</t>
+      <c r="BN21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transcend Lineage</t>
         </is>
       </c>
       <c r="HA21" t="inlineStr">
@@ -3978,6 +3918,16 @@
           <t xml:space="preserve">Rees Cast Stone Company (REECA)</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rees Cast Stone Company</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rees Cast Stone Company</t>
+        </is>
+      </c>
       <c r="U22" t="inlineStr">
         <is>
           <t xml:space="preserve">38-E</t>
@@ -3990,22 +3940,22 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mortar, Dark Chocolate, 38-E, Building Materials, Masonry, Mortar</t>
+          <t xml:space="preserve">Rees Cast Stone Company Rees Cast Stone Company, Mortar, Dark Chocolate, 38-E</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t xml:space="preserve">MORTAR</t>
+          <t xml:space="preserve">MORTAR 38-E</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dark Chocolate 38-E Mortar</t>
+          <t xml:space="preserve">Rees Cast Stone Company Dark Chocolate 38-E Mortar</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mortar, Dark Chocolate</t>
+          <t xml:space="preserve">Rees Cast Stone Company Mortar, Dark Chocolate</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -4092,7 +4042,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco Products, Inc. Satco®, Light Bulb, Incan, S3709, Electrical</t>
+          <t xml:space="preserve">Satco Products, Inc. Satco, Light Bulb, S3709, 25 W, 2700 K</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -4102,17 +4052,17 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Incan S3709 Light Bulb, 25 W, 2700 K</t>
+          <t xml:space="preserve">Satco® S3709 Light Bulb, 25 W, 2700 K</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Light Bulb, Incan, 25 W, 2700 K</t>
+          <t xml:space="preserve">Satco® Light Bulb, 25 W, 2700 K</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incan Light Bulb, 25 W, 2700 K</t>
+          <t xml:space="preserve">Light Bulb, 25 W, 2700 K</t>
         </is>
       </c>
       <c r="BC23" t="inlineStr">
@@ -4122,40 +4072,30 @@
       </c>
       <c r="BD23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Wattage</t>
         </is>
       </c>
       <c r="BE23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incan</t>
+          <t xml:space="preserve">25</t>
+        </is>
+      </c>
+      <c r="BF23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W</t>
         </is>
       </c>
       <c r="BG23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wattage</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BH23" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t xml:space="preserve">2700</t>
         </is>
       </c>
       <c r="BI23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">W</t>
-        </is>
-      </c>
-      <c r="BJ23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Color Temperature</t>
-        </is>
-      </c>
-      <c r="BK23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2700</t>
-        </is>
-      </c>
-      <c r="BL23" t="inlineStr">
         <is>
           <t xml:space="preserve">K</t>
         </is>
@@ -4204,27 +4144,27 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t xml:space="preserve">CertainTeed LLC CertainTeed®, Firelite, 653258, 4 in x 9 in</t>
+          <t xml:space="preserve">CertainTeed LLC CertainTeed, Firelite, 653258, 4 in x 9 in, Drywall</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIRELITE 4IN X 9IN</t>
+          <t xml:space="preserve">FIRELITE 4IN X 9IN DRYWALL</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t xml:space="preserve">CertainTeed® 653258 Firelite, 4 in x 9 in</t>
+          <t xml:space="preserve">CertainTeed® 653258 Firelite, 4 in x 9 in, Drywall</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t xml:space="preserve">CertainTeed® Firelite, 4 in x 9 in</t>
+          <t xml:space="preserve">CertainTeed® Firelite, 4 in x 9 in, Drywall</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Firelite, 4 in x 9 in</t>
+          <t xml:space="preserve">Firelite, 4 in x 9 in, Drywall</t>
         </is>
       </c>
       <c r="BC24" t="inlineStr">
@@ -4265,6 +4205,16 @@
       <c r="BT24" t="inlineStr">
         <is>
           <t xml:space="preserve">4 in x 9 in</t>
+        </is>
+      </c>
+      <c r="BV24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Application</t>
+        </is>
+      </c>
+      <c r="BW24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drywall</t>
         </is>
       </c>
     </row>
@@ -4326,27 +4276,27 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t xml:space="preserve">The AZEK Company AZEK®, Decking, Castle Gate Landmark, AGB15516CG</t>
+          <t xml:space="preserve">The AZEK Company AZEK, Decking, Castle Gate, AGB15516CG, 1 in x 6 in</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECKING 1IN X 6IN 16FT</t>
+          <t xml:space="preserve">DECKING 1IN X 6IN 16FT GRVD</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t xml:space="preserve">AZEK® Castle Gate Landmark AGB15516CG Decking, 1 in x 6 in, 16 ft</t>
+          <t xml:space="preserve">AZEK® Castle Gate AGB15516CG Decking, 1 in x 6 in, 16 ft, Grooved</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t xml:space="preserve">AZEK® Decking, Castle Gate Landmark, 1 in x 6 in, 16 ft</t>
+          <t xml:space="preserve">AZEK® Decking, Castle Gate, 1 in x 6 in, 16 ft, Grooved</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Castle Gate Landmark Decking, 1 in x 6 in, 16 ft</t>
+          <t xml:space="preserve">Castle Gate Decking, 1 in x 6 in, 16 ft, Grooved</t>
         </is>
       </c>
       <c r="BC25" t="inlineStr">
@@ -4381,12 +4331,22 @@
       </c>
       <c r="BJ25" t="inlineStr">
         <is>
+          <t xml:space="preserve">Edge Profile</t>
+        </is>
+      </c>
+      <c r="BK25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grooved</t>
+        </is>
+      </c>
+      <c r="BM25" t="inlineStr">
+        <is>
           <t xml:space="preserve">Series</t>
         </is>
       </c>
-      <c r="BK25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Castle Gate Landmark</t>
+      <c r="BN25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Castle Gate</t>
         </is>
       </c>
       <c r="HA25" t="inlineStr">
@@ -4453,12 +4413,12 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alliance Laundry Systems Speed Queen®, Washer, TR5006WN, Appliances</t>
+          <t xml:space="preserve">Alliance Laundry Systems Speed Queen, Washer, TR5006WN, White</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t xml:space="preserve">WASHER WH</t>
+          <t xml:space="preserve">WASHER WH TR5006WN</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
@@ -4555,7 +4515,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Signify Holding Philips®, Light Bulb, Led, 573485, Electrical</t>
+          <t xml:space="preserve">Signify Holding Philips, Light Bulb, 573485, 60 W, 5000 K, LED</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
@@ -4565,17 +4525,17 @@
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Led 573485 Light Bulb, 60 W, 5000 K, LED, A19</t>
+          <t xml:space="preserve">Philips® 573485 Light Bulb, 60 W, 5000 K, LED, A19</t>
         </is>
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philips® Light Bulb, Led, 60 W, 5000 K, LED, A19, Medium Base, 2</t>
+          <t xml:space="preserve">Philips® Light Bulb, 60 W, 5000 K, LED, A19, Medium Base, 2</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led Light Bulb, 60 W, 5000 K, LED, A19</t>
+          <t xml:space="preserve">Light Bulb, 60 W, 5000 K, LED, A19</t>
         </is>
       </c>
       <c r="BC27" t="inlineStr">
@@ -4585,80 +4545,70 @@
       </c>
       <c r="BD27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Wattage</t>
         </is>
       </c>
       <c r="BE27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led</t>
+          <t xml:space="preserve">60</t>
+        </is>
+      </c>
+      <c r="BF27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W</t>
         </is>
       </c>
       <c r="BG27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wattage</t>
+          <t xml:space="preserve">Color Temperature</t>
         </is>
       </c>
       <c r="BH27" t="inlineStr">
         <is>
-          <t xml:space="preserve">60</t>
+          <t xml:space="preserve">5000</t>
         </is>
       </c>
       <c r="BI27" t="inlineStr">
         <is>
-          <t xml:space="preserve">W</t>
+          <t xml:space="preserve">K</t>
         </is>
       </c>
       <c r="BJ27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Color Temperature</t>
+          <t xml:space="preserve">Lamp Type</t>
         </is>
       </c>
       <c r="BK27" t="inlineStr">
         <is>
-          <t xml:space="preserve">5000</t>
-        </is>
-      </c>
-      <c r="BL27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K</t>
+          <t xml:space="preserve">LED</t>
         </is>
       </c>
       <c r="BM27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamp Type</t>
+          <t xml:space="preserve">Bulb Shape</t>
         </is>
       </c>
       <c r="BN27" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED</t>
+          <t xml:space="preserve">A19</t>
         </is>
       </c>
       <c r="BP27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bulb Shape</t>
+          <t xml:space="preserve">Base Type</t>
         </is>
       </c>
       <c r="BQ27" t="inlineStr">
         <is>
-          <t xml:space="preserve">A19</t>
+          <t xml:space="preserve">Medium Base</t>
         </is>
       </c>
       <c r="BS27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base Type</t>
+          <t xml:space="preserve">Pack Quantity</t>
         </is>
       </c>
       <c r="BT27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Medium Base</t>
-        </is>
-      </c>
-      <c r="BV27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pack Quantity</t>
-        </is>
-      </c>
-      <c r="BW27" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
@@ -4677,12 +4627,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power Tool Accessories</t>
+          <t xml:space="preserve">Hand Tools</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Driver Bits</t>
+          <t xml:space="preserve">Screwdrivers</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4722,62 +4672,62 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tools &amp; Equipment&gt;Power Tool Accessories&gt;Driver Bits</t>
+          <t xml:space="preserve">Tools &amp; Equipment&gt;Hand Tools&gt;Screwdrivers</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vessel Co., Inc. Vessel®, Bit, Screwdriver Plus, 220USBP5U, Tools</t>
+          <t xml:space="preserve">Vessel Co., Inc. Vessel, Screwdriver, 220USBP5U, 5, Set</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIT 5</t>
+          <t xml:space="preserve">SCREWDRIVER 5 SET</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vessel® Screwdriver Plus 220USBP5U Bit, 5</t>
+          <t xml:space="preserve">Vessel® 220USBP5U Screwdriver, 5, Set</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vessel® Bit, Screwdriver Plus, 5</t>
+          <t xml:space="preserve">Vessel® Screwdriver, 5, Set</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Screwdriver Plus Bit, 5</t>
+          <t xml:space="preserve">Screwdriver, 5, Set</t>
         </is>
       </c>
       <c r="BC28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bit</t>
+          <t xml:space="preserve">Screwdriver</t>
         </is>
       </c>
       <c r="BD28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Pack Quantity</t>
         </is>
       </c>
       <c r="BE28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Screwdriver Plus</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="BG28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pack Quantity</t>
+          <t xml:space="preserve">Configuration</t>
         </is>
       </c>
       <c r="BH28" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">Set</t>
         </is>
       </c>
       <c r="HA28" t="inlineStr">
         <is>
-          <t xml:space="preserve">27112800</t>
+          <t xml:space="preserve">27111500</t>
         </is>
       </c>
     </row>
@@ -4819,32 +4769,32 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMT Utensili S.p.A. CMT®, Dado, 230.312.08</t>
+          <t xml:space="preserve">CMT Utensili S.p.A. CMT, Locked Dado, 230.312.08, Set</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t xml:space="preserve">DADO</t>
+          <t xml:space="preserve">LOCKED DADO SET</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMT® 230.312.08 Dado</t>
+          <t xml:space="preserve">CMT® 230.312.08 Locked Dado, Set</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMT® Dado</t>
+          <t xml:space="preserve">CMT® Locked Dado, Set</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dado</t>
+          <t xml:space="preserve">Locked Dado, Set</t>
         </is>
       </c>
       <c r="BC29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dado</t>
+          <t xml:space="preserve">Locked Dado</t>
         </is>
       </c>
       <c r="BD29" t="inlineStr">
@@ -4870,6 +4820,16 @@
       <c r="BP29" t="inlineStr">
         <is>
           <t xml:space="preserve">Pack Quantity</t>
+        </is>
+      </c>
+      <c r="BS29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Configuration</t>
+        </is>
+      </c>
+      <c r="BT29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4891,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wolf Peak International Edge Eyewear®, Safety Glasses</t>
+          <t xml:space="preserve">Wolf Peak International Edge Eyewear, Safety Glasses, Makalu Frame Polarized</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -4941,17 +4901,17 @@
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edge Eyewear® Edge Makalu Frame Polarized MK113MPAP Safety Glasses, Black</t>
+          <t xml:space="preserve">Edge Eyewear® Makalu Frame Polarized MK113MPAP Safety Glasses, Black</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edge Eyewear® Safety Glasses, Edge Makalu Frame Polarized, Black</t>
+          <t xml:space="preserve">Edge Eyewear® Safety Glasses, Makalu Frame Polarized, Black</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edge Makalu Frame Polarized Safety Glasses, Black</t>
+          <t xml:space="preserve">Makalu Frame Polarized Safety Glasses, Black</t>
         </is>
       </c>
       <c r="BC30" t="inlineStr">
@@ -4966,7 +4926,7 @@
       </c>
       <c r="BE30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edge Makalu Frame Polarized</t>
+          <t xml:space="preserve">Makalu Frame Polarized</t>
         </is>
       </c>
       <c r="BG30" t="inlineStr">
@@ -5033,12 +4993,12 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microwave, CVM517P3RD1, Appliances, Large Appliances, Microwaves</t>
+          <t xml:space="preserve">Microwave, CVM517P3RD1, Black</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t xml:space="preserve">MICROWAVE BK</t>
+          <t xml:space="preserve">MICROWAVE BK CVM517P3RD1</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
@@ -5135,32 +5095,32 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee Tool Milwaukee®, Disc, Dual Cut, 49-94-0923, Tools</t>
+          <t xml:space="preserve">Milwaukee Tool Milwaukee, Grind Disc, Dual Cut, 49-94-0923, 7/8 in</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t xml:space="preserve">DISC 6IN 1/8IN 7/8IN 6IN X 1/8IN X 7/8IN</t>
+          <t xml:space="preserve">GRIND DISC 6IN 1/8IN 7/8IN METAL</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee® Dual Cut 49-94-0923 Disc, 6 in x 1/8 in x 7/8 in, 7/8 in, 6 in, 1/8 in</t>
+          <t xml:space="preserve">Milwaukee® Dual Cut 49-94-0923 Grind Disc, 6 in x 1/8 in x 7/8 in, Metal</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee® Disc, Dual Cut, 6 in x 1/8 in x 7/8 in, 7/8 in, 6 in, 1/8 in</t>
+          <t xml:space="preserve">Milwaukee® Grind Disc, Dual Cut, 6 in x 1/8 in x 7/8 in, Metal</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dual Cut Disc, 6 in x 1/8 in x 7/8 in, 7/8 in, 6 in, 1/8 in</t>
+          <t xml:space="preserve">Dual Cut Grind Disc, 6 in x 1/8 in x 7/8 in, Metal</t>
         </is>
       </c>
       <c r="BC32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disc</t>
+          <t xml:space="preserve">Grind Disc</t>
         </is>
       </c>
       <c r="BD32" t="inlineStr">
@@ -5226,6 +5186,16 @@
       <c r="BR32" t="inlineStr">
         <is>
           <t xml:space="preserve">in</t>
+        </is>
+      </c>
+      <c r="BS32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Application</t>
+        </is>
+      </c>
+      <c r="BT32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metal</t>
         </is>
       </c>
       <c r="HA32" t="inlineStr">
@@ -5292,32 +5262,32 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leviton Manufacturing Co., Inc. Leviton®, Outlet, R02-GUAC1-0BW</t>
+          <t xml:space="preserve">Leviton Manufacturing Co., Inc. Leviton, USB Outlet, R02-GUAC1-0BW</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTLET WH 15A</t>
+          <t xml:space="preserve">USB OUTLET WH 15A</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leviton® R02-GUAC1-0BW Outlet, 15 A, White</t>
+          <t xml:space="preserve">Leviton® R02-GUAC1-0BW USB Outlet, 15 A, White</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leviton® Outlet, 15 A, White</t>
+          <t xml:space="preserve">Leviton® USB Outlet, 15 A, White</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outlet, 15 A, White</t>
+          <t xml:space="preserve">USB Outlet, 15 A, White</t>
         </is>
       </c>
       <c r="BC33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outlet</t>
+          <t xml:space="preserve">USB Outlet</t>
         </is>
       </c>
       <c r="BD33" t="inlineStr">
@@ -5409,7 +5379,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco Products, Inc. Satco®, Ceiling Light, Led, 62-1850, Electrical</t>
+          <t xml:space="preserve">Satco Products, Inc. Satco, Ceiling Light, 62-1850, 11 in, LED</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -5419,17 +5389,17 @@
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Led 62-1850 Ceiling Light, 11 in, LED</t>
+          <t xml:space="preserve">Satco® 62-1850 Ceiling Light, 11 in, LED</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Satco® Ceiling Light, Led, 11 in, LED</t>
+          <t xml:space="preserve">Satco® Ceiling Light, 11 in, LED</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led Ceiling Light, 11 in, LED</t>
+          <t xml:space="preserve">Ceiling Light, 11 in, LED</t>
         </is>
       </c>
       <c r="BC34" t="inlineStr">
@@ -5439,35 +5409,25 @@
       </c>
       <c r="BD34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Size</t>
         </is>
       </c>
       <c r="BE34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Led</t>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="BF34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">in</t>
         </is>
       </c>
       <c r="BG34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Size</t>
+          <t xml:space="preserve">Lamp Type</t>
         </is>
       </c>
       <c r="BH34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="BI34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">in</t>
-        </is>
-      </c>
-      <c r="BJ34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lamp Type</t>
-        </is>
-      </c>
-      <c r="BK34" t="inlineStr">
         <is>
           <t xml:space="preserve">LED</t>
         </is>
@@ -5536,12 +5496,12 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makita U.S.A., Inc. Makita®, Organizer, Deep Compact, T-90065</t>
+          <t xml:space="preserve">Makita U.S.A., Inc. Makita, Organizer, Deep Compact, T-90065</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORGANIZER</t>
+          <t xml:space="preserve">ORGANIZER T-90065</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
@@ -5638,12 +5598,12 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Element Electronics Element, Freezer, EUF17CDBW, Appliances, Large Appliances</t>
+          <t xml:space="preserve">Element Electronics Element, Freezer, EUF17CDBW</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREEZER</t>
+          <t xml:space="preserve">FREEZER EUF17CDBW</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
@@ -5730,12 +5690,12 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milwaukee Tool Milwaukee®, Orange, Mason Line Brd, 25459, Building Materials</t>
+          <t xml:space="preserve">Milwaukee Tool Milwaukee, Orange, Mason Line Brd, 25459, 500 ft</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORANGE 500FT</t>
+          <t xml:space="preserve">ORANGE 500FT 25459</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
@@ -5847,42 +5807,42 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE Appliances Café®, Machine, Espresso MB, C7CESAS3RD3, Appliances</t>
+          <t xml:space="preserve">GE Appliances Café, Espresso Machine, C7CESAS3RD3, Matte Black</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t xml:space="preserve">MACHINE</t>
+          <t xml:space="preserve">ESPRESSO MACHINE MATTE BLACK</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Café® Espresso MB C7CESAS3RD3 Machine</t>
+          <t xml:space="preserve">Café® C7CESAS3RD3 Espresso Machine, Matte Black</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Café® Machine, Espresso MB</t>
+          <t xml:space="preserve">Café® Espresso Machine, Matte Black</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espresso MB Machine</t>
+          <t xml:space="preserve">Espresso Machine, Matte Black</t>
         </is>
       </c>
       <c r="BC38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine</t>
+          <t xml:space="preserve">Espresso Machine</t>
         </is>
       </c>
       <c r="BD38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Color</t>
         </is>
       </c>
       <c r="BE38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espresso MB</t>
+          <t xml:space="preserve">Matte Black</t>
         </is>
       </c>
       <c r="HA38" t="inlineStr">
@@ -5949,12 +5909,12 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE Appliances GE®, Refrigerator, PGE29BYTFS, Appliances, Large Appliances</t>
+          <t xml:space="preserve">GE Appliances GE, Refrigerator, PGE29BYTFS, Stainless Steel</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t xml:space="preserve">REFRIG SST</t>
+          <t xml:space="preserve">REFRIG SST PGE29BYTFS</t>
         </is>
       </c>
       <c r="Z39" t="inlineStr">
@@ -6051,27 +6011,27 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex Company, Inc. Trex®, Decking, Biscayne Sq Edge Transcend Lineage, 543140020</t>
+          <t xml:space="preserve">Trex Company, Inc. Trex, Decking, Transcend Lineage, 543140020</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECKING 1IN X 6IN 20FT</t>
+          <t xml:space="preserve">DECKING 1IN X 6IN 20FT SQ EDG</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Biscayne Sq Edge Transcend Lineage 543140020 Decking, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Trex® Transcend Lineage 543140020 Decking, 1 in x 6 in, 20 ft, Square Edge</t>
         </is>
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trex® Decking, Biscayne Sq Edge Transcend Lineage, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Trex® Decking, Transcend Lineage, 1 in x 6 in, 20 ft, Square Edge</t>
         </is>
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscayne Sq Edge Transcend Lineage Decking, 1 in x 6 in, 20 ft</t>
+          <t xml:space="preserve">Transcend Lineage Decking, 1 in x 6 in, 20 ft, Square Edge</t>
         </is>
       </c>
       <c r="BC40" t="inlineStr">
@@ -6106,12 +6066,22 @@
       </c>
       <c r="BJ40" t="inlineStr">
         <is>
+          <t xml:space="preserve">Edge Profile</t>
+        </is>
+      </c>
+      <c r="BK40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square Edge</t>
+        </is>
+      </c>
+      <c r="BM40" t="inlineStr">
+        <is>
           <t xml:space="preserve">Series</t>
         </is>
       </c>
-      <c r="BK40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Biscayne Sq Edge Transcend Lineage</t>
+      <c r="BN40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transcend Lineage</t>
         </is>
       </c>
       <c r="HA40" t="inlineStr">
@@ -6178,7 +6148,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE Appliances GE®, Cooktop, PEP9030DTBB, Appliances, Large Appliances</t>
+          <t xml:space="preserve">GE Appliances GE, Cooktop, PEP9030DTBB, 30 in, Black</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">

</xml_diff>